<commit_message>
docs(erd): prescription_items.guidance 추가 (dbml · 입력 · FHIR 대응 · 변경 이력)
- dbml: prescription_items.guidance jsonb
- xlsx 입력 탭 38행 · FHIR 대응 탭 37행 추가, 변경 이력 v1.3 아래 상세 2행
- 요약 탭 자동 집계: 입력 필드 49→50, 신규 22→23

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V8oVyHQb3NFLeStGcY2ZQ3
</commit_message>
<xml_diff>
--- a/docs/planning/ERD_6기_5팀_v1.3.xlsx
+++ b/docs/planning/ERD_6기_5팀_v1.3.xlsx
@@ -20,12 +20,12 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'사용자'!$A$4:$N$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'입력'!$A$4:$N$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'입력'!$A$4:$N$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'분석'!$A$4:$N$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'챗봇'!$A$4:$N$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'실천·보상'!$A$4:$N$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'마스터'!$A$4:$N$106</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'FHIR 대응'!$A$5:$H$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'FHIR 대응'!$A$5:$H$84</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -876,7 +876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2155,132 +2155,128 @@
       <c r="H36" s="15" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="22" t="inlineStr">
+      <c r="A37" s="16" t="inlineStr">
         <is>
           <t>입력</t>
         </is>
       </c>
-      <c r="B37" s="37" t="inlineStr">
+      <c r="B37" s="33" t="inlineStr">
         <is>
           <t>prescription_items</t>
         </is>
       </c>
-      <c r="C37" s="21" t="inlineStr">
+      <c r="C37" s="15" t="inlineStr">
+        <is>
+          <t>guidance</t>
+        </is>
+      </c>
+      <c r="D37" s="15" t="inlineStr">
+        <is>
+          <t>MedicationRequest</t>
+        </is>
+      </c>
+      <c r="E37" s="15" t="inlineStr">
+        <is>
+          <t>MedicationRequest.dosageInstruction.patientInstruction</t>
+        </is>
+      </c>
+      <c r="F37" s="15" t="inlineStr">
+        <is>
+          <t>문장 목록 → 줄바꿈으로 이어 붙인 text</t>
+        </is>
+      </c>
+      <c r="G37" s="16" t="inlineStr">
+        <is>
+          <t>변환</t>
+        </is>
+      </c>
+      <c r="H37" s="15" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="22" t="inlineStr">
+        <is>
+          <t>입력</t>
+        </is>
+      </c>
+      <c r="B38" s="37" t="inlineStr">
+        <is>
+          <t>prescription_items</t>
+        </is>
+      </c>
+      <c r="C38" s="21" t="inlineStr">
         <is>
           <t>match_status · match_score</t>
         </is>
       </c>
-      <c r="D37" s="21" t="inlineStr">
+      <c r="D38" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E37" s="21" t="inlineStr">
+      <c r="E38" s="21" t="inlineStr">
         <is>
           <t>extension</t>
         </is>
       </c>
-      <c r="F37" s="21" t="inlineStr"/>
-      <c r="G37" s="22" t="inlineStr">
+      <c r="F38" s="21" t="inlineStr"/>
+      <c r="G38" s="22" t="inlineStr">
         <is>
           <t>확장</t>
         </is>
       </c>
-      <c r="H37" s="21" t="inlineStr">
+      <c r="H38" s="21" t="inlineStr">
         <is>
           <t>약품 매칭 상태는 내부 처리 정보</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="34" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="34" t="inlineStr">
         <is>
           <t>입력</t>
         </is>
       </c>
-      <c r="B38" s="40" t="inlineStr">
+      <c r="B39" s="40" t="inlineStr">
         <is>
           <t>prescription_item_candidates</t>
         </is>
       </c>
-      <c r="C38" s="36" t="inlineStr">
+      <c r="C39" s="36" t="inlineStr">
         <is>
           <t>(테이블)</t>
         </is>
       </c>
-      <c r="D38" s="17" t="inlineStr">
+      <c r="D39" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E38" s="36" t="inlineStr">
+      <c r="E39" s="36" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F38" s="36" t="inlineStr"/>
-      <c r="G38" s="34" t="inlineStr">
+      <c r="F39" s="36" t="inlineStr"/>
+      <c r="G39" s="34" t="inlineStr">
         <is>
           <t>FHIR 외</t>
         </is>
       </c>
-      <c r="H38" s="36" t="inlineStr">
+      <c r="H39" s="36" t="inlineStr">
         <is>
           <t>약품 매칭 후보 (내부 처리)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="16" t="inlineStr">
-        <is>
-          <t>입력</t>
-        </is>
-      </c>
-      <c r="B39" s="19" t="inlineStr">
-        <is>
-          <t>health_checkups · checkup_results</t>
-        </is>
-      </c>
-      <c r="C39" s="15" t="inlineStr">
-        <is>
-          <t>(테이블)</t>
-        </is>
-      </c>
-      <c r="D39" s="14" t="inlineStr">
-        <is>
-          <t>DiagnosticReport · Observation</t>
-        </is>
-      </c>
-      <c r="E39" s="15" t="inlineStr">
-        <is>
-          <t>Observation.code / valueQuantity</t>
-        </is>
-      </c>
-      <c r="F39" s="15" t="inlineStr">
-        <is>
-          <t>검진 항목 코드 → Observation.code</t>
-        </is>
-      </c>
-      <c r="G39" s="16" t="inlineStr">
-        <is>
-          <t>변환</t>
-        </is>
-      </c>
-      <c r="H39" s="15" t="inlineStr">
-        <is>
-          <t>보류 (REQ-015)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="16" t="inlineStr">
         <is>
-          <t>분석</t>
+          <t>입력</t>
         </is>
       </c>
       <c r="B40" s="19" t="inlineStr">
         <is>
-          <t>analyses</t>
+          <t>health_checkups · checkup_results</t>
         </is>
       </c>
       <c r="C40" s="15" t="inlineStr">
@@ -2290,17 +2286,17 @@
       </c>
       <c r="D40" s="14" t="inlineStr">
         <is>
-          <t>Task</t>
+          <t>DiagnosticReport · Observation</t>
         </is>
       </c>
       <c r="E40" s="15" t="inlineStr">
         <is>
-          <t>Task</t>
+          <t>Observation.code / valueQuantity</t>
         </is>
       </c>
       <c r="F40" s="15" t="inlineStr">
         <is>
-          <t>분석 작업 1건 = Task 1개</t>
+          <t>검진 항목 코드 → Observation.code</t>
         </is>
       </c>
       <c r="G40" s="16" t="inlineStr">
@@ -2310,7 +2306,7 @@
       </c>
       <c r="H40" s="15" t="inlineStr">
         <is>
-          <t>비동기 작업 상태를 Task로 표현</t>
+          <t>보류 (REQ-015)</t>
         </is>
       </c>
     </row>
@@ -2320,149 +2316,149 @@
           <t>분석</t>
         </is>
       </c>
-      <c r="B41" s="33" t="inlineStr">
+      <c r="B41" s="19" t="inlineStr">
         <is>
           <t>analyses</t>
         </is>
       </c>
       <c r="C41" s="15" t="inlineStr">
         <is>
+          <t>(테이블)</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="E41" s="15" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="F41" s="15" t="inlineStr">
+        <is>
+          <t>분석 작업 1건 = Task 1개</t>
+        </is>
+      </c>
+      <c r="G41" s="16" t="inlineStr">
+        <is>
+          <t>변환</t>
+        </is>
+      </c>
+      <c r="H41" s="15" t="inlineStr">
+        <is>
+          <t>비동기 작업 상태를 Task로 표현</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="16" t="inlineStr">
+        <is>
+          <t>분석</t>
+        </is>
+      </c>
+      <c r="B42" s="33" t="inlineStr">
+        <is>
+          <t>analyses</t>
+        </is>
+      </c>
+      <c r="C42" s="15" t="inlineStr">
+        <is>
           <t>status</t>
         </is>
       </c>
-      <c r="D41" s="15" t="inlineStr">
+      <c r="D42" s="15" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="E41" s="15" t="inlineStr">
+      <c r="E42" s="15" t="inlineStr">
         <is>
           <t>Task.status</t>
         </is>
       </c>
-      <c r="F41" s="15" t="inlineStr">
+      <c r="F42" s="15" t="inlineStr">
         <is>
           <t>queued → requested / running → in-progress / done → completed / failed → failed</t>
         </is>
       </c>
-      <c r="G41" s="16" t="inlineStr">
+      <c r="G42" s="16" t="inlineStr">
         <is>
           <t>변환</t>
         </is>
       </c>
-      <c r="H41" s="15" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="22" t="inlineStr">
+      <c r="H42" s="15" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="22" t="inlineStr">
         <is>
           <t>분석</t>
         </is>
       </c>
-      <c r="B42" s="37" t="inlineStr">
+      <c r="B43" s="37" t="inlineStr">
         <is>
           <t>analyses</t>
         </is>
       </c>
-      <c r="C42" s="21" t="inlineStr">
+      <c r="C43" s="21" t="inlineStr">
         <is>
           <t>current_step · failed_step · retry_count · error_code</t>
         </is>
       </c>
-      <c r="D42" s="21" t="inlineStr">
+      <c r="D43" s="21" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="E42" s="21" t="inlineStr">
+      <c r="E43" s="21" t="inlineStr">
         <is>
           <t>Task.businessStatus · Task.statusReason</t>
         </is>
       </c>
-      <c r="F42" s="21" t="inlineStr"/>
-      <c r="G42" s="22" t="inlineStr">
+      <c r="F43" s="21" t="inlineStr"/>
+      <c r="G43" s="22" t="inlineStr">
         <is>
           <t>확장</t>
         </is>
       </c>
-      <c r="H42" s="21" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="34" t="inlineStr">
+      <c r="H43" s="21" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="34" t="inlineStr">
         <is>
           <t>분석</t>
         </is>
       </c>
-      <c r="B43" s="35" t="inlineStr">
+      <c r="B44" s="35" t="inlineStr">
         <is>
           <t>analyses</t>
         </is>
       </c>
-      <c r="C43" s="36" t="inlineStr">
+      <c r="C44" s="36" t="inlineStr">
         <is>
           <t>user_birth_year</t>
         </is>
       </c>
-      <c r="D43" s="36" t="inlineStr">
+      <c r="D44" s="36" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E43" s="36" t="inlineStr">
+      <c r="E44" s="36" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F43" s="36" t="inlineStr"/>
-      <c r="G43" s="34" t="inlineStr">
+      <c r="F44" s="36" t="inlineStr"/>
+      <c r="G44" s="34" t="inlineStr">
         <is>
           <t>FHIR 외</t>
         </is>
       </c>
-      <c r="H43" s="36" t="inlineStr">
+      <c r="H44" s="36" t="inlineStr">
         <is>
           <t>분석 시점 스냅샷 (내부)</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="16" t="inlineStr">
-        <is>
-          <t>분석</t>
-        </is>
-      </c>
-      <c r="B44" s="19" t="inlineStr">
-        <is>
-          <t>analysis_prescriptions</t>
-        </is>
-      </c>
-      <c r="C44" s="15" t="inlineStr">
-        <is>
-          <t>(테이블)</t>
-        </is>
-      </c>
-      <c r="D44" s="14" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="E44" s="15" t="inlineStr">
-        <is>
-          <t>Task.input</t>
-        </is>
-      </c>
-      <c r="F44" s="15" t="inlineStr">
-        <is>
-          <t>valueReference = MedicationRequest</t>
-        </is>
-      </c>
-      <c r="G44" s="16" t="inlineStr">
-        <is>
-          <t>변환</t>
-        </is>
-      </c>
-      <c r="H44" s="15" t="inlineStr">
-        <is>
-          <t>분석에 넣은 처방 목록</t>
         </is>
       </c>
     </row>
@@ -2474,7 +2470,7 @@
       </c>
       <c r="B45" s="19" t="inlineStr">
         <is>
-          <t>analysis_diseases</t>
+          <t>analysis_prescriptions</t>
         </is>
       </c>
       <c r="C45" s="15" t="inlineStr">
@@ -2484,21 +2480,29 @@
       </c>
       <c r="D45" s="14" t="inlineStr">
         <is>
-          <t>Condition</t>
+          <t>Task</t>
         </is>
       </c>
       <c r="E45" s="15" t="inlineStr">
         <is>
-          <t>Condition</t>
-        </is>
-      </c>
-      <c r="F45" s="15" t="inlineStr"/>
+          <t>Task.input</t>
+        </is>
+      </c>
+      <c r="F45" s="15" t="inlineStr">
+        <is>
+          <t>valueReference = MedicationRequest</t>
+        </is>
+      </c>
       <c r="G45" s="16" t="inlineStr">
         <is>
           <t>변환</t>
         </is>
       </c>
-      <c r="H45" s="15" t="inlineStr"/>
+      <c r="H45" s="15" t="inlineStr">
+        <is>
+          <t>분석에 넣은 처방 목록</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="16" t="inlineStr">
@@ -2506,123 +2510,115 @@
           <t>분석</t>
         </is>
       </c>
-      <c r="B46" s="33" t="inlineStr">
+      <c r="B46" s="19" t="inlineStr">
         <is>
           <t>analysis_diseases</t>
         </is>
       </c>
       <c r="C46" s="15" t="inlineStr">
         <is>
+          <t>(테이블)</t>
+        </is>
+      </c>
+      <c r="D46" s="14" t="inlineStr">
+        <is>
+          <t>Condition</t>
+        </is>
+      </c>
+      <c r="E46" s="15" t="inlineStr">
+        <is>
+          <t>Condition</t>
+        </is>
+      </c>
+      <c r="F46" s="15" t="inlineStr"/>
+      <c r="G46" s="16" t="inlineStr">
+        <is>
+          <t>변환</t>
+        </is>
+      </c>
+      <c r="H46" s="15" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="16" t="inlineStr">
+        <is>
+          <t>분석</t>
+        </is>
+      </c>
+      <c r="B47" s="33" t="inlineStr">
+        <is>
+          <t>analysis_diseases</t>
+        </is>
+      </c>
+      <c r="C47" s="15" t="inlineStr">
+        <is>
           <t>origin</t>
         </is>
       </c>
-      <c r="D46" s="15" t="inlineStr">
+      <c r="D47" s="15" t="inlineStr">
         <is>
           <t>Condition</t>
         </is>
       </c>
-      <c r="E46" s="15" t="inlineStr">
+      <c r="E47" s="15" t="inlineStr">
         <is>
           <t>Condition.asserter</t>
         </is>
       </c>
-      <c r="F46" s="15" t="inlineStr">
+      <c r="F47" s="15" t="inlineStr">
         <is>
           <t>prescription → 처방전에서 옴 / user → asserter = Patient (직접 선택)</t>
         </is>
       </c>
-      <c r="G46" s="16" t="inlineStr">
+      <c r="G47" s="16" t="inlineStr">
         <is>
           <t>변환</t>
         </is>
       </c>
-      <c r="H46" s="15" t="inlineStr">
+      <c r="H47" s="15" t="inlineStr">
         <is>
           <t>누가 주장한 질환인지 구분</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="30" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="30" t="inlineStr">
         <is>
           <t>분석</t>
         </is>
       </c>
-      <c r="B47" s="38" t="inlineStr">
+      <c r="B48" s="38" t="inlineStr">
         <is>
           <t>analysis_warnings</t>
         </is>
       </c>
-      <c r="C47" s="32" t="inlineStr">
+      <c r="C48" s="32" t="inlineStr">
         <is>
           <t>(테이블)</t>
         </is>
       </c>
-      <c r="D47" s="39" t="inlineStr">
+      <c r="D48" s="39" t="inlineStr">
         <is>
           <t>DetectedIssue</t>
         </is>
       </c>
-      <c r="E47" s="32" t="inlineStr">
+      <c r="E48" s="32" t="inlineStr">
         <is>
           <t>DetectedIssue</t>
         </is>
       </c>
-      <c r="F47" s="32" t="inlineStr">
+      <c r="F48" s="32" t="inlineStr">
         <is>
           <t>경고 1건 = DetectedIssue 1개</t>
         </is>
       </c>
-      <c r="G47" s="30" t="inlineStr">
+      <c r="G48" s="30" t="inlineStr">
         <is>
           <t>일치</t>
         </is>
       </c>
-      <c r="H47" s="32" t="inlineStr">
+      <c r="H48" s="32" t="inlineStr">
         <is>
           <t>FHIR에 "약물 문제 감지" 전용 리소스가 있음 — 가장 잘 맞는 부분</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="16" t="inlineStr">
-        <is>
-          <t>분석</t>
-        </is>
-      </c>
-      <c r="B48" s="33" t="inlineStr">
-        <is>
-          <t>analysis_warnings</t>
-        </is>
-      </c>
-      <c r="C48" s="15" t="inlineStr">
-        <is>
-          <t>warning_type</t>
-        </is>
-      </c>
-      <c r="D48" s="15" t="inlineStr">
-        <is>
-          <t>DetectedIssue</t>
-        </is>
-      </c>
-      <c r="E48" s="15" t="inlineStr">
-        <is>
-          <t>DetectedIssue.code</t>
-        </is>
-      </c>
-      <c r="F48" s="15" t="inlineStr">
-        <is>
-          <t>interaction → DRG / duplicate_* → DUPTHPY / dose_exceed → DOSEHIGH / age → AGE / elderly · pregnancy · polypharmacy → 자체 코드</t>
-        </is>
-      </c>
-      <c r="G48" s="16" t="inlineStr">
-        <is>
-          <t>변환</t>
-        </is>
-      </c>
-      <c r="H48" s="15" t="inlineStr">
-        <is>
-          <t>HL7 v3 ActCode 후보 — 구현 시 코드 확인 필요</t>
         </is>
       </c>
     </row>
@@ -2639,68 +2635,72 @@
       </c>
       <c r="C49" s="15" t="inlineStr">
         <is>
+          <t>warning_type</t>
+        </is>
+      </c>
+      <c r="D49" s="15" t="inlineStr">
+        <is>
+          <t>DetectedIssue</t>
+        </is>
+      </c>
+      <c r="E49" s="15" t="inlineStr">
+        <is>
+          <t>DetectedIssue.code</t>
+        </is>
+      </c>
+      <c r="F49" s="15" t="inlineStr">
+        <is>
+          <t>interaction → DRG / duplicate_* → DUPTHPY / dose_exceed → DOSEHIGH / age → AGE / elderly · pregnancy · polypharmacy → 자체 코드</t>
+        </is>
+      </c>
+      <c r="G49" s="16" t="inlineStr">
+        <is>
+          <t>변환</t>
+        </is>
+      </c>
+      <c r="H49" s="15" t="inlineStr">
+        <is>
+          <t>HL7 v3 ActCode 후보 — 구현 시 코드 확인 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="16" t="inlineStr">
+        <is>
+          <t>분석</t>
+        </is>
+      </c>
+      <c r="B50" s="33" t="inlineStr">
+        <is>
+          <t>analysis_warnings</t>
+        </is>
+      </c>
+      <c r="C50" s="15" t="inlineStr">
+        <is>
           <t>severity</t>
         </is>
       </c>
-      <c r="D49" s="15" t="inlineStr">
+      <c r="D50" s="15" t="inlineStr">
         <is>
           <t>DetectedIssue</t>
         </is>
       </c>
-      <c r="E49" s="15" t="inlineStr">
+      <c r="E50" s="15" t="inlineStr">
         <is>
           <t>DetectedIssue.severity</t>
         </is>
       </c>
-      <c r="F49" s="15" t="inlineStr">
+      <c r="F50" s="15" t="inlineStr">
         <is>
           <t>danger → high / caution → moderate / info → low</t>
         </is>
       </c>
-      <c r="G49" s="16" t="inlineStr">
+      <c r="G50" s="16" t="inlineStr">
         <is>
           <t>변환</t>
         </is>
       </c>
-      <c r="H49" s="15" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="30" t="inlineStr">
-        <is>
-          <t>분석</t>
-        </is>
-      </c>
-      <c r="B50" s="31" t="inlineStr">
-        <is>
-          <t>analysis_warnings</t>
-        </is>
-      </c>
-      <c r="C50" s="32" t="inlineStr">
-        <is>
-          <t>item_id_a · item_id_b</t>
-        </is>
-      </c>
-      <c r="D50" s="32" t="inlineStr">
-        <is>
-          <t>DetectedIssue</t>
-        </is>
-      </c>
-      <c r="E50" s="32" t="inlineStr">
-        <is>
-          <t>DetectedIssue.implicated</t>
-        </is>
-      </c>
-      <c r="F50" s="32" t="inlineStr">
-        <is>
-          <t>Reference(MedicationRequest) 2개</t>
-        </is>
-      </c>
-      <c r="G50" s="30" t="inlineStr">
-        <is>
-          <t>일치</t>
-        </is>
-      </c>
-      <c r="H50" s="32" t="inlineStr"/>
+      <c r="H50" s="15" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="30" t="inlineStr">
@@ -2715,142 +2715,142 @@
       </c>
       <c r="C51" s="32" t="inlineStr">
         <is>
+          <t>item_id_a · item_id_b</t>
+        </is>
+      </c>
+      <c r="D51" s="32" t="inlineStr">
+        <is>
+          <t>DetectedIssue</t>
+        </is>
+      </c>
+      <c r="E51" s="32" t="inlineStr">
+        <is>
+          <t>DetectedIssue.implicated</t>
+        </is>
+      </c>
+      <c r="F51" s="32" t="inlineStr">
+        <is>
+          <t>Reference(MedicationRequest) 2개</t>
+        </is>
+      </c>
+      <c r="G51" s="30" t="inlineStr">
+        <is>
+          <t>일치</t>
+        </is>
+      </c>
+      <c r="H51" s="32" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="30" t="inlineStr">
+        <is>
+          <t>분석</t>
+        </is>
+      </c>
+      <c r="B52" s="31" t="inlineStr">
+        <is>
+          <t>analysis_warnings</t>
+        </is>
+      </c>
+      <c r="C52" s="32" t="inlineStr">
+        <is>
           <t>reason</t>
         </is>
       </c>
-      <c r="D51" s="32" t="inlineStr">
+      <c r="D52" s="32" t="inlineStr">
         <is>
           <t>DetectedIssue</t>
         </is>
       </c>
-      <c r="E51" s="32" t="inlineStr">
+      <c r="E52" s="32" t="inlineStr">
         <is>
           <t>DetectedIssue.detail</t>
         </is>
       </c>
-      <c r="F51" s="32" t="inlineStr">
+      <c r="F52" s="32" t="inlineStr">
         <is>
           <t>DUR 금기 사유 원문</t>
         </is>
       </c>
-      <c r="G51" s="30" t="inlineStr">
+      <c r="G52" s="30" t="inlineStr">
         <is>
           <t>일치</t>
         </is>
       </c>
-      <c r="H51" s="32" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="16" t="inlineStr">
+      <c r="H52" s="32" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="16" t="inlineStr">
         <is>
           <t>분석</t>
         </is>
       </c>
-      <c r="B52" s="33" t="inlineStr">
+      <c r="B53" s="33" t="inlineStr">
         <is>
           <t>analysis_warnings</t>
         </is>
       </c>
-      <c r="C52" s="15" t="inlineStr">
+      <c r="C53" s="15" t="inlineStr">
         <is>
           <t>source · notice_date</t>
         </is>
       </c>
-      <c r="D52" s="15" t="inlineStr">
+      <c r="D53" s="15" t="inlineStr">
         <is>
           <t>DetectedIssue</t>
         </is>
       </c>
-      <c r="E52" s="15" t="inlineStr">
+      <c r="E53" s="15" t="inlineStr">
         <is>
           <t>DetectedIssue.reference</t>
         </is>
       </c>
-      <c r="F52" s="15" t="inlineStr">
+      <c r="F53" s="15" t="inlineStr">
         <is>
           <t>식약처 고시 출처</t>
         </is>
       </c>
-      <c r="G52" s="16" t="inlineStr">
+      <c r="G53" s="16" t="inlineStr">
         <is>
           <t>변환</t>
         </is>
       </c>
-      <c r="H52" s="15" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="22" t="inlineStr">
+      <c r="H53" s="15" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="22" t="inlineStr">
         <is>
           <t>분석</t>
         </is>
       </c>
-      <c r="B53" s="37" t="inlineStr">
+      <c r="B54" s="37" t="inlineStr">
         <is>
           <t>analysis_warnings</t>
         </is>
       </c>
-      <c r="C53" s="21" t="inlineStr">
+      <c r="C54" s="21" t="inlineStr">
         <is>
           <t>summary · daily_total · max_daily</t>
         </is>
       </c>
-      <c r="D53" s="21" t="inlineStr">
+      <c r="D54" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E53" s="21" t="inlineStr">
+      <c r="E54" s="21" t="inlineStr">
         <is>
           <t>extension</t>
         </is>
       </c>
-      <c r="F53" s="21" t="inlineStr"/>
-      <c r="G53" s="22" t="inlineStr">
+      <c r="F54" s="21" t="inlineStr"/>
+      <c r="G54" s="22" t="inlineStr">
         <is>
           <t>확장</t>
         </is>
       </c>
-      <c r="H53" s="21" t="inlineStr">
+      <c r="H54" s="21" t="inlineStr">
         <is>
           <t>화면 문장 · 용량 계산값</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="34" t="inlineStr">
-        <is>
-          <t>분석</t>
-        </is>
-      </c>
-      <c r="B54" s="40" t="inlineStr">
-        <is>
-          <t>guides</t>
-        </is>
-      </c>
-      <c r="C54" s="36" t="inlineStr">
-        <is>
-          <t>(테이블)</t>
-        </is>
-      </c>
-      <c r="D54" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E54" s="36" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F54" s="36" t="inlineStr"/>
-      <c r="G54" s="34" t="inlineStr">
-        <is>
-          <t>FHIR 외</t>
-        </is>
-      </c>
-      <c r="H54" s="36" t="inlineStr">
-        <is>
-          <t>AI 생성 안내문 (의료 기록 아님). 필요하면 DocumentReference로 보관</t>
         </is>
       </c>
     </row>
@@ -2862,7 +2862,7 @@
       </c>
       <c r="B55" s="40" t="inlineStr">
         <is>
-          <t>feedbacks</t>
+          <t>guides</t>
         </is>
       </c>
       <c r="C55" s="36" t="inlineStr">
@@ -2888,19 +2888,19 @@
       </c>
       <c r="H55" s="36" t="inlineStr">
         <is>
-          <t>서비스 피드백</t>
+          <t>AI 생성 안내문 (의료 기록 아님). 필요하면 DocumentReference로 보관</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="34" t="inlineStr">
         <is>
-          <t>챗봇</t>
+          <t>분석</t>
         </is>
       </c>
       <c r="B56" s="40" t="inlineStr">
         <is>
-          <t>chat_sessions</t>
+          <t>feedbacks</t>
         </is>
       </c>
       <c r="C56" s="36" t="inlineStr">
@@ -2926,45 +2926,45 @@
       </c>
       <c r="H56" s="36" t="inlineStr">
         <is>
+          <t>서비스 피드백</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="34" t="inlineStr">
+        <is>
+          <t>챗봇</t>
+        </is>
+      </c>
+      <c r="B57" s="40" t="inlineStr">
+        <is>
+          <t>chat_sessions</t>
+        </is>
+      </c>
+      <c r="C57" s="36" t="inlineStr">
+        <is>
+          <t>(테이블)</t>
+        </is>
+      </c>
+      <c r="D57" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E57" s="36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F57" s="36" t="inlineStr"/>
+      <c r="G57" s="34" t="inlineStr">
+        <is>
+          <t>FHIR 외</t>
+        </is>
+      </c>
+      <c r="H57" s="36" t="inlineStr">
+        <is>
           <t>대화 묶음 (내부)</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="16" t="inlineStr">
-        <is>
-          <t>챗봇</t>
-        </is>
-      </c>
-      <c r="B57" s="19" t="inlineStr">
-        <is>
-          <t>chat_messages</t>
-        </is>
-      </c>
-      <c r="C57" s="15" t="inlineStr">
-        <is>
-          <t>(테이블)</t>
-        </is>
-      </c>
-      <c r="D57" s="14" t="inlineStr">
-        <is>
-          <t>Communication</t>
-        </is>
-      </c>
-      <c r="E57" s="15" t="inlineStr">
-        <is>
-          <t>Communication</t>
-        </is>
-      </c>
-      <c r="F57" s="15" t="inlineStr"/>
-      <c r="G57" s="16" t="inlineStr">
-        <is>
-          <t>변환</t>
-        </is>
-      </c>
-      <c r="H57" s="15" t="inlineStr">
-        <is>
-          <t>의료 기록으로 보관할 필요가 생길 때만</t>
         </is>
       </c>
     </row>
@@ -2974,24 +2974,24 @@
           <t>챗봇</t>
         </is>
       </c>
-      <c r="B58" s="33" t="inlineStr">
+      <c r="B58" s="19" t="inlineStr">
         <is>
           <t>chat_messages</t>
         </is>
       </c>
       <c r="C58" s="15" t="inlineStr">
         <is>
-          <t>role · content · created_at</t>
-        </is>
-      </c>
-      <c r="D58" s="15" t="inlineStr">
+          <t>(테이블)</t>
+        </is>
+      </c>
+      <c r="D58" s="14" t="inlineStr">
         <is>
           <t>Communication</t>
         </is>
       </c>
       <c r="E58" s="15" t="inlineStr">
         <is>
-          <t>Communication.sender · payload.contentString · sent</t>
+          <t>Communication</t>
         </is>
       </c>
       <c r="F58" s="15" t="inlineStr"/>
@@ -3000,83 +3000,83 @@
           <t>변환</t>
         </is>
       </c>
-      <c r="H58" s="15" t="inlineStr"/>
+      <c r="H58" s="15" t="inlineStr">
+        <is>
+          <t>의료 기록으로 보관할 필요가 생길 때만</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="16" t="inlineStr">
         <is>
+          <t>챗봇</t>
+        </is>
+      </c>
+      <c r="B59" s="33" t="inlineStr">
+        <is>
+          <t>chat_messages</t>
+        </is>
+      </c>
+      <c r="C59" s="15" t="inlineStr">
+        <is>
+          <t>role · content · created_at</t>
+        </is>
+      </c>
+      <c r="D59" s="15" t="inlineStr">
+        <is>
+          <t>Communication</t>
+        </is>
+      </c>
+      <c r="E59" s="15" t="inlineStr">
+        <is>
+          <t>Communication.sender · payload.contentString · sent</t>
+        </is>
+      </c>
+      <c r="F59" s="15" t="inlineStr"/>
+      <c r="G59" s="16" t="inlineStr">
+        <is>
+          <t>변환</t>
+        </is>
+      </c>
+      <c r="H59" s="15" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="16" t="inlineStr">
+        <is>
           <t>실천·보상</t>
         </is>
       </c>
-      <c r="B59" s="19" t="inlineStr">
+      <c r="B60" s="19" t="inlineStr">
         <is>
           <t>recommendations</t>
         </is>
       </c>
-      <c r="C59" s="15" t="inlineStr">
+      <c r="C60" s="15" t="inlineStr">
         <is>
           <t>(테이블)</t>
         </is>
       </c>
-      <c r="D59" s="14" t="inlineStr">
+      <c r="D60" s="14" t="inlineStr">
         <is>
           <t>CarePlan</t>
         </is>
       </c>
-      <c r="E59" s="15" t="inlineStr">
+      <c r="E60" s="15" t="inlineStr">
         <is>
           <t>CarePlan.activity</t>
         </is>
       </c>
-      <c r="F59" s="15" t="inlineStr">
+      <c r="F60" s="15" t="inlineStr">
         <is>
           <t>추천 1개 = activity 1개 (status = not-started)</t>
         </is>
       </c>
-      <c r="G59" s="16" t="inlineStr">
+      <c r="G60" s="16" t="inlineStr">
         <is>
           <t>변환</t>
         </is>
       </c>
-      <c r="H59" s="15" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="30" t="inlineStr">
-        <is>
-          <t>실천·보상</t>
-        </is>
-      </c>
-      <c r="B60" s="38" t="inlineStr">
-        <is>
-          <t>habit_goals</t>
-        </is>
-      </c>
-      <c r="C60" s="32" t="inlineStr">
-        <is>
-          <t>(테이블)</t>
-        </is>
-      </c>
-      <c r="D60" s="39" t="inlineStr">
-        <is>
-          <t>Goal</t>
-        </is>
-      </c>
-      <c r="E60" s="32" t="inlineStr">
-        <is>
-          <t>Goal</t>
-        </is>
-      </c>
-      <c r="F60" s="32" t="inlineStr"/>
-      <c r="G60" s="30" t="inlineStr">
-        <is>
-          <t>일치</t>
-        </is>
-      </c>
-      <c r="H60" s="32" t="inlineStr">
-        <is>
-          <t>FHIR Goal = 환자 건강 목표</t>
-        </is>
-      </c>
+      <c r="H60" s="15" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="30" t="inlineStr">
@@ -3084,24 +3084,24 @@
           <t>실천·보상</t>
         </is>
       </c>
-      <c r="B61" s="31" t="inlineStr">
+      <c r="B61" s="38" t="inlineStr">
         <is>
           <t>habit_goals</t>
         </is>
       </c>
       <c r="C61" s="32" t="inlineStr">
         <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="D61" s="32" t="inlineStr">
+          <t>(테이블)</t>
+        </is>
+      </c>
+      <c r="D61" s="39" t="inlineStr">
         <is>
           <t>Goal</t>
         </is>
       </c>
       <c r="E61" s="32" t="inlineStr">
         <is>
-          <t>Goal.description.text</t>
+          <t>Goal</t>
         </is>
       </c>
       <c r="F61" s="32" t="inlineStr"/>
@@ -3110,7 +3110,11 @@
           <t>일치</t>
         </is>
       </c>
-      <c r="H61" s="32" t="inlineStr"/>
+      <c r="H61" s="32" t="inlineStr">
+        <is>
+          <t>FHIR Goal = 환자 건강 목표</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="30" t="inlineStr">
@@ -3125,7 +3129,7 @@
       </c>
       <c r="C62" s="32" t="inlineStr">
         <is>
-          <t>target_value · unit</t>
+          <t>title</t>
         </is>
       </c>
       <c r="D62" s="32" t="inlineStr">
@@ -3135,7 +3139,7 @@
       </c>
       <c r="E62" s="32" t="inlineStr">
         <is>
-          <t>Goal.target.detailQuantity</t>
+          <t>Goal.description.text</t>
         </is>
       </c>
       <c r="F62" s="32" t="inlineStr"/>
@@ -3159,7 +3163,7 @@
       </c>
       <c r="C63" s="32" t="inlineStr">
         <is>
-          <t>start_date · end_date</t>
+          <t>target_value · unit</t>
         </is>
       </c>
       <c r="D63" s="32" t="inlineStr">
@@ -3169,7 +3173,7 @@
       </c>
       <c r="E63" s="32" t="inlineStr">
         <is>
-          <t>Goal.startDate · Goal.target.dueDate</t>
+          <t>Goal.target.detailQuantity</t>
         </is>
       </c>
       <c r="F63" s="32" t="inlineStr"/>
@@ -3181,42 +3185,38 @@
       <c r="H63" s="32" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="16" t="inlineStr">
+      <c r="A64" s="30" t="inlineStr">
         <is>
           <t>실천·보상</t>
         </is>
       </c>
-      <c r="B64" s="33" t="inlineStr">
+      <c r="B64" s="31" t="inlineStr">
         <is>
           <t>habit_goals</t>
         </is>
       </c>
-      <c r="C64" s="15" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="D64" s="15" t="inlineStr">
+      <c r="C64" s="32" t="inlineStr">
+        <is>
+          <t>start_date · end_date</t>
+        </is>
+      </c>
+      <c r="D64" s="32" t="inlineStr">
         <is>
           <t>Goal</t>
         </is>
       </c>
-      <c r="E64" s="15" t="inlineStr">
-        <is>
-          <t>Goal.lifecycleStatus</t>
-        </is>
-      </c>
-      <c r="F64" s="15" t="inlineStr">
-        <is>
-          <t>active → active / ended → completed</t>
-        </is>
-      </c>
-      <c r="G64" s="16" t="inlineStr">
-        <is>
-          <t>변환</t>
-        </is>
-      </c>
-      <c r="H64" s="15" t="inlineStr"/>
+      <c r="E64" s="32" t="inlineStr">
+        <is>
+          <t>Goal.startDate · Goal.target.dueDate</t>
+        </is>
+      </c>
+      <c r="F64" s="32" t="inlineStr"/>
+      <c r="G64" s="30" t="inlineStr">
+        <is>
+          <t>일치</t>
+        </is>
+      </c>
+      <c r="H64" s="32" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="16" t="inlineStr">
@@ -3224,29 +3224,29 @@
           <t>실천·보상</t>
         </is>
       </c>
-      <c r="B65" s="19" t="inlineStr">
-        <is>
-          <t>habit_records</t>
+      <c r="B65" s="33" t="inlineStr">
+        <is>
+          <t>habit_goals</t>
         </is>
       </c>
       <c r="C65" s="15" t="inlineStr">
         <is>
-          <t>(테이블)</t>
-        </is>
-      </c>
-      <c r="D65" s="14" t="inlineStr">
-        <is>
-          <t>Observation</t>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D65" s="15" t="inlineStr">
+        <is>
+          <t>Goal</t>
         </is>
       </c>
       <c r="E65" s="15" t="inlineStr">
         <is>
-          <t>Observation</t>
+          <t>Goal.lifecycleStatus</t>
         </is>
       </c>
       <c r="F65" s="15" t="inlineStr">
         <is>
-          <t>기록 1건 = Observation 1개 (focus = Goal)</t>
+          <t>active → active / ended → completed</t>
         </is>
       </c>
       <c r="G65" s="16" t="inlineStr">
@@ -3262,105 +3262,109 @@
           <t>실천·보상</t>
         </is>
       </c>
-      <c r="B66" s="33" t="inlineStr">
+      <c r="B66" s="19" t="inlineStr">
         <is>
           <t>habit_records</t>
         </is>
       </c>
       <c r="C66" s="15" t="inlineStr">
         <is>
+          <t>(테이블)</t>
+        </is>
+      </c>
+      <c r="D66" s="14" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="E66" s="15" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="F66" s="15" t="inlineStr">
+        <is>
+          <t>기록 1건 = Observation 1개 (focus = Goal)</t>
+        </is>
+      </c>
+      <c r="G66" s="16" t="inlineStr">
+        <is>
+          <t>변환</t>
+        </is>
+      </c>
+      <c r="H66" s="15" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="16" t="inlineStr">
+        <is>
+          <t>실천·보상</t>
+        </is>
+      </c>
+      <c r="B67" s="33" t="inlineStr">
+        <is>
+          <t>habit_records</t>
+        </is>
+      </c>
+      <c r="C67" s="15" t="inlineStr">
+        <is>
           <t>value · completed · record_date</t>
         </is>
       </c>
-      <c r="D66" s="15" t="inlineStr">
+      <c r="D67" s="15" t="inlineStr">
         <is>
           <t>Observation</t>
         </is>
       </c>
-      <c r="E66" s="15" t="inlineStr">
+      <c r="E67" s="15" t="inlineStr">
         <is>
           <t>Observation.valueQuantity / valueBoolean · effectiveDateTime</t>
         </is>
       </c>
-      <c r="F66" s="15" t="inlineStr"/>
-      <c r="G66" s="16" t="inlineStr">
+      <c r="F67" s="15" t="inlineStr"/>
+      <c r="G67" s="16" t="inlineStr">
         <is>
           <t>변환</t>
         </is>
       </c>
-      <c r="H66" s="15" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="34" t="inlineStr">
+      <c r="H67" s="15" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="34" t="inlineStr">
         <is>
           <t>실천·보상</t>
         </is>
       </c>
-      <c r="B67" s="40" t="inlineStr">
+      <c r="B68" s="40" t="inlineStr">
         <is>
           <t>rewards</t>
         </is>
       </c>
-      <c r="C67" s="36" t="inlineStr">
+      <c r="C68" s="36" t="inlineStr">
         <is>
           <t>(테이블)</t>
         </is>
       </c>
-      <c r="D67" s="17" t="inlineStr">
+      <c r="D68" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E67" s="36" t="inlineStr">
+      <c r="E68" s="36" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F67" s="36" t="inlineStr"/>
-      <c r="G67" s="34" t="inlineStr">
+      <c r="F68" s="36" t="inlineStr"/>
+      <c r="G68" s="34" t="inlineStr">
         <is>
           <t>FHIR 외</t>
         </is>
       </c>
-      <c r="H67" s="36" t="inlineStr">
+      <c r="H68" s="36" t="inlineStr">
         <is>
           <t>포인트 (서비스 보상)</t>
         </is>
       </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="16" t="inlineStr">
-        <is>
-          <t>마스터</t>
-        </is>
-      </c>
-      <c r="B68" s="19" t="inlineStr">
-        <is>
-          <t>drug_products</t>
-        </is>
-      </c>
-      <c r="C68" s="15" t="inlineStr">
-        <is>
-          <t>(테이블)</t>
-        </is>
-      </c>
-      <c r="D68" s="14" t="inlineStr">
-        <is>
-          <t>Medication</t>
-        </is>
-      </c>
-      <c r="E68" s="15" t="inlineStr">
-        <is>
-          <t>Medication</t>
-        </is>
-      </c>
-      <c r="F68" s="15" t="inlineStr"/>
-      <c r="G68" s="16" t="inlineStr">
-        <is>
-          <t>변환</t>
-        </is>
-      </c>
-      <c r="H68" s="15" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="16" t="inlineStr">
@@ -3368,31 +3372,27 @@
           <t>마스터</t>
         </is>
       </c>
-      <c r="B69" s="33" t="inlineStr">
+      <c r="B69" s="19" t="inlineStr">
         <is>
           <t>drug_products</t>
         </is>
       </c>
       <c r="C69" s="15" t="inlineStr">
         <is>
-          <t>edi_code</t>
-        </is>
-      </c>
-      <c r="D69" s="15" t="inlineStr">
+          <t>(테이블)</t>
+        </is>
+      </c>
+      <c r="D69" s="14" t="inlineStr">
         <is>
           <t>Medication</t>
         </is>
       </c>
       <c r="E69" s="15" t="inlineStr">
         <is>
-          <t>Medication.code.coding</t>
-        </is>
-      </c>
-      <c r="F69" s="15" t="inlineStr">
-        <is>
-          <t>system = 심평원 EDI 제품코드</t>
-        </is>
-      </c>
+          <t>Medication</t>
+        </is>
+      </c>
+      <c r="F69" s="15" t="inlineStr"/>
       <c r="G69" s="16" t="inlineStr">
         <is>
           <t>변환</t>
@@ -3413,7 +3413,7 @@
       </c>
       <c r="C70" s="15" t="inlineStr">
         <is>
-          <t>ingr_code</t>
+          <t>edi_code</t>
         </is>
       </c>
       <c r="D70" s="15" t="inlineStr">
@@ -3423,12 +3423,12 @@
       </c>
       <c r="E70" s="15" t="inlineStr">
         <is>
-          <t>Medication.ingredient.itemCodeableConcept</t>
+          <t>Medication.code.coding</t>
         </is>
       </c>
       <c r="F70" s="15" t="inlineStr">
         <is>
-          <t>system = 심평원 주성분코드</t>
+          <t>system = 심평원 EDI 제품코드</t>
         </is>
       </c>
       <c r="G70" s="16" t="inlineStr">
@@ -3451,20 +3451,24 @@
       </c>
       <c r="C71" s="15" t="inlineStr">
         <is>
-          <t>entp_name</t>
+          <t>ingr_code</t>
         </is>
       </c>
       <c r="D71" s="15" t="inlineStr">
         <is>
-          <t>Organization</t>
+          <t>Medication</t>
         </is>
       </c>
       <c r="E71" s="15" t="inlineStr">
         <is>
-          <t>Medication.manufacturer → Organization.name</t>
-        </is>
-      </c>
-      <c r="F71" s="15" t="inlineStr"/>
+          <t>Medication.ingredient.itemCodeableConcept</t>
+        </is>
+      </c>
+      <c r="F71" s="15" t="inlineStr">
+        <is>
+          <t>system = 심평원 주성분코드</t>
+        </is>
+      </c>
       <c r="G71" s="16" t="inlineStr">
         <is>
           <t>변환</t>
@@ -3485,17 +3489,17 @@
       </c>
       <c r="C72" s="15" t="inlineStr">
         <is>
-          <t>spec_value · spec_unit</t>
+          <t>entp_name</t>
         </is>
       </c>
       <c r="D72" s="15" t="inlineStr">
         <is>
-          <t>Medication</t>
+          <t>Organization</t>
         </is>
       </c>
       <c r="E72" s="15" t="inlineStr">
         <is>
-          <t>Medication.ingredient.strength</t>
+          <t>Medication.manufacturer → Organization.name</t>
         </is>
       </c>
       <c r="F72" s="15" t="inlineStr"/>
@@ -3512,24 +3516,24 @@
           <t>마스터</t>
         </is>
       </c>
-      <c r="B73" s="19" t="inlineStr">
-        <is>
-          <t>drug_ingredients</t>
+      <c r="B73" s="33" t="inlineStr">
+        <is>
+          <t>drug_products</t>
         </is>
       </c>
       <c r="C73" s="15" t="inlineStr">
         <is>
-          <t>(테이블)</t>
-        </is>
-      </c>
-      <c r="D73" s="14" t="inlineStr">
-        <is>
-          <t>Substance</t>
+          <t>spec_value · spec_unit</t>
+        </is>
+      </c>
+      <c r="D73" s="15" t="inlineStr">
+        <is>
+          <t>Medication</t>
         </is>
       </c>
       <c r="E73" s="15" t="inlineStr">
         <is>
-          <t>Substance.code</t>
+          <t>Medication.ingredient.strength</t>
         </is>
       </c>
       <c r="F73" s="15" t="inlineStr"/>
@@ -3548,7 +3552,7 @@
       </c>
       <c r="B74" s="19" t="inlineStr">
         <is>
-          <t>drug_details</t>
+          <t>drug_ingredients</t>
         </is>
       </c>
       <c r="C74" s="15" t="inlineStr">
@@ -3558,29 +3562,21 @@
       </c>
       <c r="D74" s="14" t="inlineStr">
         <is>
-          <t>MedicationKnowledge</t>
+          <t>Substance</t>
         </is>
       </c>
       <c r="E74" s="15" t="inlineStr">
         <is>
-          <t>MedicationKnowledge</t>
-        </is>
-      </c>
-      <c r="F74" s="15" t="inlineStr">
-        <is>
-          <t>효능효과 · 용법용량 · 주의사항</t>
-        </is>
-      </c>
+          <t>Substance.code</t>
+        </is>
+      </c>
+      <c r="F74" s="15" t="inlineStr"/>
       <c r="G74" s="16" t="inlineStr">
         <is>
           <t>변환</t>
         </is>
       </c>
-      <c r="H74" s="15" t="inlineStr">
-        <is>
-          <t>RAG 검색 원문</t>
-        </is>
-      </c>
+      <c r="H74" s="15" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="16" t="inlineStr">
@@ -3590,7 +3586,7 @@
       </c>
       <c r="B75" s="19" t="inlineStr">
         <is>
-          <t>dur_interaction · dur_interaction_exception</t>
+          <t>drug_details</t>
         </is>
       </c>
       <c r="C75" s="15" t="inlineStr">
@@ -3600,17 +3596,17 @@
       </c>
       <c r="D75" s="14" t="inlineStr">
         <is>
-          <t>ClinicalUseDefinition (R5)</t>
+          <t>MedicationKnowledge</t>
         </is>
       </c>
       <c r="E75" s="15" t="inlineStr">
         <is>
-          <t>ClinicalUseDefinition.interaction</t>
+          <t>MedicationKnowledge</t>
         </is>
       </c>
       <c r="F75" s="15" t="inlineStr">
         <is>
-          <t>type = interaction</t>
+          <t>효능효과 · 용법용량 · 주의사항</t>
         </is>
       </c>
       <c r="G75" s="16" t="inlineStr">
@@ -3620,7 +3616,7 @@
       </c>
       <c r="H75" s="15" t="inlineStr">
         <is>
-          <t>R4에는 전용 리소스 없음 — R5 참고</t>
+          <t>RAG 검색 원문</t>
         </is>
       </c>
     </row>
@@ -3632,7 +3628,7 @@
       </c>
       <c r="B76" s="19" t="inlineStr">
         <is>
-          <t>dur_elderly · dur_age_limit · dur_pregnancy</t>
+          <t>dur_interaction · dur_interaction_exception</t>
         </is>
       </c>
       <c r="C76" s="15" t="inlineStr">
@@ -3647,12 +3643,12 @@
       </c>
       <c r="E76" s="15" t="inlineStr">
         <is>
-          <t>ClinicalUseDefinition.contraindication</t>
+          <t>ClinicalUseDefinition.interaction</t>
         </is>
       </c>
       <c r="F76" s="15" t="inlineStr">
         <is>
-          <t>type = contraindication, population = 나이 · 임부</t>
+          <t>type = interaction</t>
         </is>
       </c>
       <c r="G76" s="16" t="inlineStr">
@@ -3662,7 +3658,7 @@
       </c>
       <c r="H76" s="15" t="inlineStr">
         <is>
-          <t>R5 참고</t>
+          <t>R4에는 전용 리소스 없음 — R5 참고</t>
         </is>
       </c>
     </row>
@@ -3674,111 +3670,115 @@
       </c>
       <c r="B77" s="19" t="inlineStr">
         <is>
+          <t>dur_elderly · dur_age_limit · dur_pregnancy</t>
+        </is>
+      </c>
+      <c r="C77" s="15" t="inlineStr">
+        <is>
+          <t>(테이블)</t>
+        </is>
+      </c>
+      <c r="D77" s="14" t="inlineStr">
+        <is>
+          <t>ClinicalUseDefinition (R5)</t>
+        </is>
+      </c>
+      <c r="E77" s="15" t="inlineStr">
+        <is>
+          <t>ClinicalUseDefinition.contraindication</t>
+        </is>
+      </c>
+      <c r="F77" s="15" t="inlineStr">
+        <is>
+          <t>type = contraindication, population = 나이 · 임부</t>
+        </is>
+      </c>
+      <c r="G77" s="16" t="inlineStr">
+        <is>
+          <t>변환</t>
+        </is>
+      </c>
+      <c r="H77" s="15" t="inlineStr">
+        <is>
+          <t>R5 참고</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="16" t="inlineStr">
+        <is>
+          <t>마스터</t>
+        </is>
+      </c>
+      <c r="B78" s="19" t="inlineStr">
+        <is>
           <t>dur_dose_limit</t>
         </is>
       </c>
-      <c r="C77" s="15" t="inlineStr">
+      <c r="C78" s="15" t="inlineStr">
         <is>
           <t>(테이블)</t>
         </is>
       </c>
-      <c r="D77" s="14" t="inlineStr">
+      <c r="D78" s="14" t="inlineStr">
         <is>
           <t>MedicationKnowledge</t>
         </is>
       </c>
-      <c r="E77" s="15" t="inlineStr">
+      <c r="E78" s="15" t="inlineStr">
         <is>
           <t>MedicationKnowledge.administrationGuidelines.dosage</t>
         </is>
       </c>
-      <c r="F77" s="15" t="inlineStr">
+      <c r="F78" s="15" t="inlineStr">
         <is>
           <t>1일 최대 투여량</t>
         </is>
       </c>
-      <c r="G77" s="16" t="inlineStr">
+      <c r="G78" s="16" t="inlineStr">
         <is>
           <t>변환</t>
         </is>
       </c>
-      <c r="H77" s="15" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="34" t="inlineStr">
+      <c r="H78" s="15" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="34" t="inlineStr">
         <is>
           <t>마스터</t>
         </is>
       </c>
-      <c r="B78" s="40" t="inlineStr">
+      <c r="B79" s="40" t="inlineStr">
         <is>
           <t>dup_ingredient · dup_efficacy</t>
         </is>
       </c>
-      <c r="C78" s="36" t="inlineStr">
+      <c r="C79" s="36" t="inlineStr">
         <is>
           <t>(테이블)</t>
         </is>
       </c>
-      <c r="D78" s="17" t="inlineStr">
+      <c r="D79" s="17" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E78" s="36" t="inlineStr">
+      <c r="E79" s="36" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F78" s="36" t="inlineStr"/>
-      <c r="G78" s="34" t="inlineStr">
+      <c r="F79" s="36" t="inlineStr"/>
+      <c r="G79" s="34" t="inlineStr">
         <is>
           <t>FHIR 외</t>
         </is>
       </c>
-      <c r="H78" s="36" t="inlineStr">
+      <c r="H79" s="36" t="inlineStr">
         <is>
           <t>국내 DUR 중복 점검 규칙</t>
         </is>
       </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="16" t="inlineStr">
-        <is>
-          <t>마스터</t>
-        </is>
-      </c>
-      <c r="B79" s="19" t="inlineStr">
-        <is>
-          <t>diseases</t>
-        </is>
-      </c>
-      <c r="C79" s="15" t="inlineStr">
-        <is>
-          <t>(테이블)</t>
-        </is>
-      </c>
-      <c r="D79" s="14" t="inlineStr">
-        <is>
-          <t>CodeSystem</t>
-        </is>
-      </c>
-      <c r="E79" s="15" t="inlineStr">
-        <is>
-          <t>CodeSystem.concept</t>
-        </is>
-      </c>
-      <c r="F79" s="15" t="inlineStr">
-        <is>
-          <t>KCD 상병 코드 목록</t>
-        </is>
-      </c>
-      <c r="G79" s="16" t="inlineStr">
-        <is>
-          <t>변환</t>
-        </is>
-      </c>
-      <c r="H79" s="15" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="16" t="inlineStr">
@@ -3788,7 +3788,7 @@
       </c>
       <c r="B80" s="19" t="inlineStr">
         <is>
-          <t>checkup_items</t>
+          <t>diseases</t>
         </is>
       </c>
       <c r="C80" s="15" t="inlineStr">
@@ -3808,7 +3808,7 @@
       </c>
       <c r="F80" s="15" t="inlineStr">
         <is>
-          <t>건강검진 검사항목 코드 목록</t>
+          <t>KCD 상병 코드 목록</t>
         </is>
       </c>
       <c r="G80" s="16" t="inlineStr">
@@ -3816,11 +3816,7 @@
           <t>변환</t>
         </is>
       </c>
-      <c r="H80" s="15" t="inlineStr">
-        <is>
-          <t>보류</t>
-        </is>
-      </c>
+      <c r="H80" s="15" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="16" t="inlineStr">
@@ -3830,7 +3826,7 @@
       </c>
       <c r="B81" s="19" t="inlineStr">
         <is>
-          <t>lifestyle_guides · lifestyle_guide_actions · lifestyle_medication_links</t>
+          <t>checkup_items</t>
         </is>
       </c>
       <c r="C81" s="15" t="inlineStr">
@@ -3840,15 +3836,19 @@
       </c>
       <c r="D81" s="14" t="inlineStr">
         <is>
-          <t>PlanDefinition</t>
+          <t>CodeSystem</t>
         </is>
       </c>
       <c r="E81" s="15" t="inlineStr">
         <is>
-          <t>PlanDefinition.action</t>
-        </is>
-      </c>
-      <c r="F81" s="15" t="inlineStr"/>
+          <t>CodeSystem.concept</t>
+        </is>
+      </c>
+      <c r="F81" s="15" t="inlineStr">
+        <is>
+          <t>건강검진 검사항목 코드 목록</t>
+        </is>
+      </c>
       <c r="G81" s="16" t="inlineStr">
         <is>
           <t>변환</t>
@@ -3856,7 +3856,7 @@
       </c>
       <c r="H81" s="15" t="inlineStr">
         <is>
-          <t>자체 생활습관 지식 베이스. 실천 항목 1개 = PlanDefinition.action 1개</t>
+          <t>보류</t>
         </is>
       </c>
     </row>
@@ -3868,80 +3868,118 @@
       </c>
       <c r="B82" s="19" t="inlineStr">
         <is>
+          <t>lifestyle_guides · lifestyle_guide_actions · lifestyle_medication_links</t>
+        </is>
+      </c>
+      <c r="C82" s="15" t="inlineStr">
+        <is>
+          <t>(테이블)</t>
+        </is>
+      </c>
+      <c r="D82" s="14" t="inlineStr">
+        <is>
+          <t>PlanDefinition</t>
+        </is>
+      </c>
+      <c r="E82" s="15" t="inlineStr">
+        <is>
+          <t>PlanDefinition.action</t>
+        </is>
+      </c>
+      <c r="F82" s="15" t="inlineStr"/>
+      <c r="G82" s="16" t="inlineStr">
+        <is>
+          <t>변환</t>
+        </is>
+      </c>
+      <c r="H82" s="15" t="inlineStr">
+        <is>
+          <t>자체 생활습관 지식 베이스. 실천 항목 1개 = PlanDefinition.action 1개</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="16" t="inlineStr">
+        <is>
+          <t>마스터</t>
+        </is>
+      </c>
+      <c r="B83" s="19" t="inlineStr">
+        <is>
           <t>lifestyle_guide_sources</t>
         </is>
       </c>
-      <c r="C82" s="15" t="inlineStr">
+      <c r="C83" s="15" t="inlineStr">
         <is>
           <t>(테이블)</t>
         </is>
       </c>
-      <c r="D82" s="14" t="inlineStr">
+      <c r="D83" s="14" t="inlineStr">
         <is>
           <t>DocumentReference / Citation (R5)</t>
         </is>
       </c>
-      <c r="E82" s="15" t="inlineStr">
+      <c r="E83" s="15" t="inlineStr">
         <is>
           <t>PlanDefinition.relatedArtifact</t>
         </is>
       </c>
-      <c r="F82" s="15" t="inlineStr">
+      <c r="F83" s="15" t="inlineStr">
         <is>
           <t>type = citation · display = 문서명 · url · citation = 기관 · 발행일</t>
         </is>
       </c>
-      <c r="G82" s="16" t="inlineStr">
+      <c r="G83" s="16" t="inlineStr">
         <is>
           <t>변환</t>
         </is>
       </c>
-      <c r="H82" s="15" t="inlineStr">
+      <c r="H83" s="15" t="inlineStr">
         <is>
           <t>v1.2 · R4는 relatedArtifact로 출처 표시</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" s="22" t="inlineStr">
+    <row r="84">
+      <c r="A84" s="22" t="inlineStr">
         <is>
           <t>마스터</t>
         </is>
       </c>
-      <c r="B83" s="37" t="inlineStr">
+      <c r="B84" s="37" t="inlineStr">
         <is>
           <t>lifestyle_medication_links</t>
         </is>
       </c>
-      <c r="C83" s="21" t="inlineStr">
+      <c r="C84" s="21" t="inlineStr">
         <is>
           <t>requires_clinician · goal_eligible</t>
         </is>
       </c>
-      <c r="D83" s="21" t="inlineStr">
+      <c r="D84" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E83" s="21" t="inlineStr">
+      <c r="E84" s="21" t="inlineStr">
         <is>
           <t>extension</t>
         </is>
       </c>
-      <c r="F83" s="21" t="inlineStr"/>
-      <c r="G83" s="22" t="inlineStr">
+      <c r="F84" s="21" t="inlineStr"/>
+      <c r="G84" s="22" t="inlineStr">
         <is>
           <t>확장</t>
         </is>
       </c>
-      <c r="H83" s="21" t="inlineStr">
+      <c r="H84" s="21" t="inlineStr">
         <is>
           <t>v1.2 · 서비스 표시 규칙</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:H83"/>
+  <autoFilter ref="A5:H84"/>
   <dataValidations count="1">
     <dataValidation sqref="G6:G300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"일치,변환,확장,FHIR 외"</formula1>
@@ -3957,7 +3995,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E153"/>
+  <dimension ref="A1:E155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6914,6 +6952,44 @@
         </is>
       </c>
       <c r="E153" s="10" t="n"/>
+    </row>
+    <row r="154" hidden="1" outlineLevel="1">
+      <c r="A154" s="10" t="n"/>
+      <c r="B154" s="10" t="inlineStr">
+        <is>
+          <t>입력 / prescription_items.guidance — 필드 추가</t>
+        </is>
+      </c>
+      <c r="C154" s="10" t="inlineStr">
+        <is>
+          <t>(없음)</t>
+        </is>
+      </c>
+      <c r="D154" s="10" t="inlineStr">
+        <is>
+          <t>guidance jsonb · N · 약봉투 약 카드에 약국이 인쇄한 복약 안내 문장 목록 (마스킹 후 저장, 없으면 null)</t>
+        </is>
+      </c>
+      <c r="E154" s="10" t="n"/>
+    </row>
+    <row r="155" hidden="1" outlineLevel="1">
+      <c r="A155" s="10" t="n"/>
+      <c r="B155" s="10" t="inlineStr">
+        <is>
+          <t>FHIR 대응 탭 — prescription_items.guidance 행 추가</t>
+        </is>
+      </c>
+      <c r="C155" s="10" t="inlineStr">
+        <is>
+          <t>78행</t>
+        </is>
+      </c>
+      <c r="D155" s="10" t="inlineStr">
+        <is>
+          <t>79행 — guidance → MedicationRequest.dosageInstruction.patientInstruction (변환: 문장 목록 → 줄바꿈으로 이어 붙인 text)</t>
+        </is>
+      </c>
+      <c r="E155" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -8284,7 +8360,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N53"/>
+  <dimension ref="A1:N54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10278,68 +10354,60 @@
       <c r="N37" s="21" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="23" t="inlineStr">
-        <is>
-          <t>prescription_item_candidates</t>
-        </is>
-      </c>
-      <c r="B38" s="24" t="inlineStr">
-        <is>
-          <t>약품 매칭 후보</t>
-        </is>
-      </c>
-      <c r="C38" s="24" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="D38" s="24" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="E38" s="24" t="inlineStr">
-        <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="F38" s="25" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="G38" s="24" t="n"/>
-      <c r="H38" s="25" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I38" s="24" t="n"/>
-      <c r="J38" s="24" t="inlineStr">
-        <is>
-          <t>코드 구현 맞춤 — Tortoise는 복합 PK를 지원하지 않아 id를 PK로 두고 원래 PK 두 칸은 unique로</t>
-        </is>
-      </c>
-      <c r="K38" s="24" t="inlineStr">
-        <is>
-          <t>OC-02 · O-3</t>
-        </is>
-      </c>
-      <c r="L38" s="25" t="inlineStr">
+      <c r="A38" s="20" t="inlineStr">
+        <is>
+          <t>prescription_items</t>
+        </is>
+      </c>
+      <c r="B38" s="21" t="inlineStr">
+        <is>
+          <t>처방 약품</t>
+        </is>
+      </c>
+      <c r="C38" s="21" t="inlineStr">
+        <is>
+          <t>guidance</t>
+        </is>
+      </c>
+      <c r="D38" s="21" t="inlineStr">
+        <is>
+          <t>약국 인쇄 복약 안내</t>
+        </is>
+      </c>
+      <c r="E38" s="21" t="inlineStr">
+        <is>
+          <t>jsonb</t>
+        </is>
+      </c>
+      <c r="F38" s="22" t="n"/>
+      <c r="G38" s="21" t="n"/>
+      <c r="H38" s="22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I38" s="21" t="n"/>
+      <c r="J38" s="21" t="inlineStr">
+        <is>
+          <t>약봉투만 채움, 마스킹 후 저장. 없으면 null</t>
+        </is>
+      </c>
+      <c r="K38" s="21" t="inlineStr">
+        <is>
+          <t>OC-02 · O-2 · O-3</t>
+        </is>
+      </c>
+      <c r="L38" s="22" t="inlineStr">
         <is>
           <t>신규</t>
         </is>
       </c>
-      <c r="M38" s="25" t="inlineStr">
+      <c r="M38" s="22" t="inlineStr">
         <is>
           <t>v1.3</t>
         </is>
       </c>
-      <c r="N38" s="24" t="inlineStr">
-        <is>
-          <t>v1.0 신규 🟡 채연 확인 · OC-02 후보 목록. 매칭 정확도(1순위 적중률 · 5순위 내 포함률) 측정에 필요 · v1.3 id PK + (item_id, rank) UQ · v1.3 edi_code · item_seq 중 하나는 꼭 있음</t>
-        </is>
-      </c>
+      <c r="N38" s="21" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="23" t="inlineStr">
@@ -10354,12 +10422,12 @@
       </c>
       <c r="C39" s="24" t="inlineStr">
         <is>
-          <t>item_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="D39" s="24" t="inlineStr">
         <is>
-          <t>처방 약품 ID</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="E39" s="24" t="inlineStr">
@@ -10369,21 +10437,21 @@
       </c>
       <c r="F39" s="25" t="inlineStr">
         <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="G39" s="24" t="inlineStr">
-        <is>
-          <t>prescription_items.id</t>
-        </is>
-      </c>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="G39" s="24" t="n"/>
       <c r="H39" s="25" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
       <c r="I39" s="24" t="n"/>
-      <c r="J39" s="24" t="n"/>
+      <c r="J39" s="24" t="inlineStr">
+        <is>
+          <t>코드 구현 맞춤 — Tortoise는 복합 PK를 지원하지 않아 id를 PK로 두고 원래 PK 두 칸은 unique로</t>
+        </is>
+      </c>
       <c r="K39" s="24" t="inlineStr">
         <is>
           <t>OC-02 · O-3</t>
@@ -10399,7 +10467,11 @@
           <t>v1.3</t>
         </is>
       </c>
-      <c r="N39" s="24" t="n"/>
+      <c r="N39" s="24" t="inlineStr">
+        <is>
+          <t>v1.0 신규 🟡 채연 확인 · OC-02 후보 목록. 매칭 정확도(1순위 적중률 · 5순위 내 포함률) 측정에 필요 · v1.3 id PK + (item_id, rank) UQ · v1.3 edi_code · item_seq 중 하나는 꼭 있음</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="23" t="inlineStr">
@@ -10414,32 +10486,36 @@
       </c>
       <c r="C40" s="24" t="inlineStr">
         <is>
-          <t>rank</t>
+          <t>item_id</t>
         </is>
       </c>
       <c r="D40" s="24" t="inlineStr">
         <is>
-          <t>순위</t>
+          <t>처방 약품 ID</t>
         </is>
       </c>
       <c r="E40" s="24" t="inlineStr">
         <is>
-          <t>smallint</t>
-        </is>
-      </c>
-      <c r="F40" s="25" t="n"/>
-      <c r="G40" s="24" t="n"/>
+          <t>bigint</t>
+        </is>
+      </c>
+      <c r="F40" s="25" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="G40" s="24" t="inlineStr">
+        <is>
+          <t>prescription_items.id</t>
+        </is>
+      </c>
       <c r="H40" s="25" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
       <c r="I40" s="24" t="n"/>
-      <c r="J40" s="24" t="inlineStr">
-        <is>
-          <t>(item_id, rank) UQ</t>
-        </is>
-      </c>
+      <c r="J40" s="24" t="n"/>
       <c r="K40" s="24" t="inlineStr">
         <is>
           <t>OC-02 · O-3</t>
@@ -10470,38 +10546,30 @@
       </c>
       <c r="C41" s="24" t="inlineStr">
         <is>
-          <t>edi_code</t>
+          <t>rank</t>
         </is>
       </c>
       <c r="D41" s="24" t="inlineStr">
         <is>
-          <t>EDI 제품코드</t>
+          <t>순위</t>
         </is>
       </c>
       <c r="E41" s="24" t="inlineStr">
         <is>
-          <t>varchar(9)</t>
-        </is>
-      </c>
-      <c r="F41" s="25" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="G41" s="24" t="inlineStr">
-        <is>
-          <t>drug_products.edi_code</t>
-        </is>
-      </c>
+          <t>smallint</t>
+        </is>
+      </c>
+      <c r="F41" s="25" t="n"/>
+      <c r="G41" s="24" t="n"/>
       <c r="H41" s="25" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I41" s="24" t="n"/>
       <c r="J41" s="24" t="inlineStr">
         <is>
-          <t>급여목록에 있는 약 (없는 약은 item_seq) — 둘 중 하나는 꼭 있음</t>
+          <t>(item_id, rank) UQ</t>
         </is>
       </c>
       <c r="K41" s="24" t="inlineStr">
@@ -10534,12 +10602,12 @@
       </c>
       <c r="C42" s="24" t="inlineStr">
         <is>
-          <t>item_seq</t>
+          <t>edi_code</t>
         </is>
       </c>
       <c r="D42" s="24" t="inlineStr">
         <is>
-          <t>품목기준코드</t>
+          <t>EDI 제품코드</t>
         </is>
       </c>
       <c r="E42" s="24" t="inlineStr">
@@ -10554,7 +10622,7 @@
       </c>
       <c r="G42" s="24" t="inlineStr">
         <is>
-          <t>drug_details.item_seq</t>
+          <t>drug_products.edi_code</t>
         </is>
       </c>
       <c r="H42" s="25" t="inlineStr">
@@ -10565,7 +10633,7 @@
       <c r="I42" s="24" t="n"/>
       <c r="J42" s="24" t="inlineStr">
         <is>
-          <t>급여목록에 없는 약 — edi_code가 없을 때 채움</t>
+          <t>급여목록에 있는 약 (없는 약은 item_seq) — 둘 중 하나는 꼭 있음</t>
         </is>
       </c>
       <c r="K42" s="24" t="inlineStr">
@@ -10598,104 +10666,108 @@
       </c>
       <c r="C43" s="24" t="inlineStr">
         <is>
+          <t>item_seq</t>
+        </is>
+      </c>
+      <c r="D43" s="24" t="inlineStr">
+        <is>
+          <t>품목기준코드</t>
+        </is>
+      </c>
+      <c r="E43" s="24" t="inlineStr">
+        <is>
+          <t>varchar(9)</t>
+        </is>
+      </c>
+      <c r="F43" s="25" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="G43" s="24" t="inlineStr">
+        <is>
+          <t>drug_details.item_seq</t>
+        </is>
+      </c>
+      <c r="H43" s="25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I43" s="24" t="n"/>
+      <c r="J43" s="24" t="inlineStr">
+        <is>
+          <t>급여목록에 없는 약 — edi_code가 없을 때 채움</t>
+        </is>
+      </c>
+      <c r="K43" s="24" t="inlineStr">
+        <is>
+          <t>OC-02 · O-3</t>
+        </is>
+      </c>
+      <c r="L43" s="25" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="M43" s="25" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="N43" s="24" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="23" t="inlineStr">
+        <is>
+          <t>prescription_item_candidates</t>
+        </is>
+      </c>
+      <c r="B44" s="24" t="inlineStr">
+        <is>
+          <t>약품 매칭 후보</t>
+        </is>
+      </c>
+      <c r="C44" s="24" t="inlineStr">
+        <is>
           <t>score</t>
         </is>
       </c>
-      <c r="D43" s="24" t="inlineStr">
+      <c r="D44" s="24" t="inlineStr">
         <is>
           <t>매칭 점수</t>
         </is>
       </c>
-      <c r="E43" s="24" t="inlineStr">
+      <c r="E44" s="24" t="inlineStr">
         <is>
           <t>decimal(5,4)</t>
         </is>
       </c>
-      <c r="F43" s="25" t="n"/>
-      <c r="G43" s="24" t="n"/>
-      <c r="H43" s="25" t="inlineStr">
+      <c r="F44" s="25" t="n"/>
+      <c r="G44" s="24" t="n"/>
+      <c r="H44" s="25" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I43" s="24" t="n"/>
-      <c r="J43" s="24" t="n"/>
-      <c r="K43" s="24" t="inlineStr">
+      <c r="I44" s="24" t="n"/>
+      <c r="J44" s="24" t="n"/>
+      <c r="K44" s="24" t="inlineStr">
         <is>
           <t>OC-02 · O-3</t>
         </is>
       </c>
-      <c r="L43" s="25" t="inlineStr">
+      <c r="L44" s="25" t="inlineStr">
         <is>
           <t>신규</t>
         </is>
       </c>
-      <c r="M43" s="25" t="inlineStr">
+      <c r="M44" s="25" t="inlineStr">
         <is>
           <t>v1.0</t>
         </is>
       </c>
-      <c r="N43" s="24" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="19" t="inlineStr">
-        <is>
-          <t>health_checkups</t>
-        </is>
-      </c>
-      <c r="B44" s="15" t="inlineStr">
-        <is>
-          <t>건강검진 (보류)</t>
-        </is>
-      </c>
-      <c r="C44" s="15" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="D44" s="15" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="E44" s="15" t="inlineStr">
-        <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="F44" s="16" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="G44" s="15" t="n"/>
-      <c r="H44" s="16" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I44" s="15" t="n"/>
-      <c r="J44" s="15" t="n"/>
-      <c r="K44" s="15" t="inlineStr">
-        <is>
-          <t>REQ-015</t>
-        </is>
-      </c>
-      <c r="L44" s="16" t="inlineStr">
-        <is>
-          <t>기존</t>
-        </is>
-      </c>
-      <c r="M44" s="16" t="inlineStr">
-        <is>
-          <t>v0.1</t>
-        </is>
-      </c>
-      <c r="N44" s="15" t="inlineStr">
-        <is>
-          <t>보류 (REQ-015 · 멘토링 확인 후 결정)</t>
-        </is>
-      </c>
+      <c r="N44" s="24" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="19" t="inlineStr">
@@ -10710,12 +10782,12 @@
       </c>
       <c r="C45" s="15" t="inlineStr">
         <is>
-          <t>user_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="D45" s="15" t="inlineStr">
         <is>
-          <t>사용자 ID</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="E45" s="15" t="inlineStr">
@@ -10725,14 +10797,10 @@
       </c>
       <c r="F45" s="16" t="inlineStr">
         <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="G45" s="15" t="inlineStr">
-        <is>
-          <t>users.id</t>
-        </is>
-      </c>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="G45" s="15" t="n"/>
       <c r="H45" s="16" t="inlineStr">
         <is>
           <t>Y</t>
@@ -10755,7 +10823,11 @@
           <t>v0.1</t>
         </is>
       </c>
-      <c r="N45" s="15" t="n"/>
+      <c r="N45" s="15" t="inlineStr">
+        <is>
+          <t>보류 (REQ-015 · 멘토링 확인 후 결정)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="19" t="inlineStr">
@@ -10770,24 +10842,32 @@
       </c>
       <c r="C46" s="15" t="inlineStr">
         <is>
-          <t>checkup_date</t>
+          <t>user_id</t>
         </is>
       </c>
       <c r="D46" s="15" t="inlineStr">
         <is>
-          <t>검진일</t>
+          <t>사용자 ID</t>
         </is>
       </c>
       <c r="E46" s="15" t="inlineStr">
         <is>
-          <t>date</t>
-        </is>
-      </c>
-      <c r="F46" s="16" t="n"/>
-      <c r="G46" s="15" t="n"/>
+          <t>bigint</t>
+        </is>
+      </c>
+      <c r="F46" s="16" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="G46" s="15" t="inlineStr">
+        <is>
+          <t>users.id</t>
+        </is>
+      </c>
       <c r="H46" s="16" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I46" s="15" t="n"/>
@@ -10822,17 +10902,17 @@
       </c>
       <c r="C47" s="15" t="inlineStr">
         <is>
-          <t>ocr_raw_text</t>
+          <t>checkup_date</t>
         </is>
       </c>
       <c r="D47" s="15" t="inlineStr">
         <is>
-          <t>OCR 원문</t>
+          <t>검진일</t>
         </is>
       </c>
       <c r="E47" s="15" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>date</t>
         </is>
       </c>
       <c r="F47" s="16" t="n"/>
@@ -10874,17 +10954,17 @@
       </c>
       <c r="C48" s="15" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>ocr_raw_text</t>
         </is>
       </c>
       <c r="D48" s="15" t="inlineStr">
         <is>
-          <t>생성 일시</t>
+          <t>OCR 원문</t>
         </is>
       </c>
       <c r="E48" s="15" t="inlineStr">
         <is>
-          <t>timestamp</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F48" s="16" t="n"/>
@@ -10894,11 +10974,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I48" s="15" t="inlineStr">
-        <is>
-          <t>now()</t>
-        </is>
-      </c>
+      <c r="I48" s="15" t="n"/>
       <c r="J48" s="15" t="n"/>
       <c r="K48" s="15" t="inlineStr">
         <is>
@@ -10920,41 +10996,41 @@
     <row r="49">
       <c r="A49" s="19" t="inlineStr">
         <is>
-          <t>checkup_results</t>
+          <t>health_checkups</t>
         </is>
       </c>
       <c r="B49" s="15" t="inlineStr">
         <is>
-          <t>건강검진 결과 (보류)</t>
+          <t>건강검진 (보류)</t>
         </is>
       </c>
       <c r="C49" s="15" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="D49" s="15" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>생성 일시</t>
         </is>
       </c>
       <c r="E49" s="15" t="inlineStr">
         <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="F49" s="16" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
+          <t>timestamp</t>
+        </is>
+      </c>
+      <c r="F49" s="16" t="n"/>
       <c r="G49" s="15" t="n"/>
       <c r="H49" s="16" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I49" s="15" t="n"/>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I49" s="15" t="inlineStr">
+        <is>
+          <t>now()</t>
+        </is>
+      </c>
       <c r="J49" s="15" t="n"/>
       <c r="K49" s="15" t="inlineStr">
         <is>
@@ -10971,11 +11047,7 @@
           <t>v0.1</t>
         </is>
       </c>
-      <c r="N49" s="15" t="inlineStr">
-        <is>
-          <t>보류 (REQ-015)</t>
-        </is>
-      </c>
+      <c r="N49" s="15" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="19" t="inlineStr">
@@ -10990,12 +11062,12 @@
       </c>
       <c r="C50" s="15" t="inlineStr">
         <is>
-          <t>checkup_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="D50" s="15" t="inlineStr">
         <is>
-          <t>건강검진 ID</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="E50" s="15" t="inlineStr">
@@ -11005,14 +11077,10 @@
       </c>
       <c r="F50" s="16" t="inlineStr">
         <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="G50" s="15" t="inlineStr">
-        <is>
-          <t>health_checkups.id</t>
-        </is>
-      </c>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="G50" s="15" t="n"/>
       <c r="H50" s="16" t="inlineStr">
         <is>
           <t>Y</t>
@@ -11035,67 +11103,71 @@
           <t>v0.1</t>
         </is>
       </c>
-      <c r="N50" s="15" t="n"/>
+      <c r="N50" s="15" t="inlineStr">
+        <is>
+          <t>보류 (REQ-015)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="20" t="inlineStr">
+      <c r="A51" s="19" t="inlineStr">
         <is>
           <t>checkup_results</t>
         </is>
       </c>
-      <c r="B51" s="21" t="inlineStr">
+      <c r="B51" s="15" t="inlineStr">
         <is>
           <t>건강검진 결과 (보류)</t>
         </is>
       </c>
-      <c r="C51" s="21" t="inlineStr">
-        <is>
-          <t>item_code</t>
-        </is>
-      </c>
-      <c r="D51" s="21" t="inlineStr">
-        <is>
-          <t>검사 항목 코드</t>
-        </is>
-      </c>
-      <c r="E51" s="21" t="inlineStr">
-        <is>
-          <t>varchar(8)</t>
-        </is>
-      </c>
-      <c r="F51" s="22" t="inlineStr">
+      <c r="C51" s="15" t="inlineStr">
+        <is>
+          <t>checkup_id</t>
+        </is>
+      </c>
+      <c r="D51" s="15" t="inlineStr">
+        <is>
+          <t>건강검진 ID</t>
+        </is>
+      </c>
+      <c r="E51" s="15" t="inlineStr">
+        <is>
+          <t>bigint</t>
+        </is>
+      </c>
+      <c r="F51" s="16" t="inlineStr">
         <is>
           <t>FK</t>
         </is>
       </c>
-      <c r="G51" s="21" t="inlineStr">
-        <is>
-          <t>checkup_items.code</t>
-        </is>
-      </c>
-      <c r="H51" s="22" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I51" s="21" t="n"/>
-      <c r="J51" s="21" t="n"/>
-      <c r="K51" s="21" t="inlineStr">
+      <c r="G51" s="15" t="inlineStr">
+        <is>
+          <t>health_checkups.id</t>
+        </is>
+      </c>
+      <c r="H51" s="16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I51" s="15" t="n"/>
+      <c r="J51" s="15" t="n"/>
+      <c r="K51" s="15" t="inlineStr">
         <is>
           <t>REQ-015</t>
         </is>
       </c>
-      <c r="L51" s="22" t="inlineStr">
-        <is>
-          <t>수정</t>
-        </is>
-      </c>
-      <c r="M51" s="22" t="inlineStr">
-        <is>
-          <t>v1.0</t>
-        </is>
-      </c>
-      <c r="N51" s="21" t="n"/>
+      <c r="L51" s="16" t="inlineStr">
+        <is>
+          <t>기존</t>
+        </is>
+      </c>
+      <c r="M51" s="16" t="inlineStr">
+        <is>
+          <t>v0.1</t>
+        </is>
+      </c>
+      <c r="N51" s="15" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="20" t="inlineStr">
@@ -11110,21 +11182,29 @@
       </c>
       <c r="C52" s="21" t="inlineStr">
         <is>
-          <t>value_num</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="D52" s="21" t="inlineStr">
         <is>
-          <t>결과 수치</t>
+          <t>검사 항목 코드</t>
         </is>
       </c>
       <c r="E52" s="21" t="inlineStr">
         <is>
-          <t>decimal(12,3)</t>
-        </is>
-      </c>
-      <c r="F52" s="22" t="n"/>
-      <c r="G52" s="21" t="n"/>
+          <t>varchar(8)</t>
+        </is>
+      </c>
+      <c r="F52" s="22" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="G52" s="21" t="inlineStr">
+        <is>
+          <t>checkup_items.code</t>
+        </is>
+      </c>
       <c r="H52" s="22" t="inlineStr">
         <is>
           <t>N</t>
@@ -11162,17 +11242,17 @@
       </c>
       <c r="C53" s="21" t="inlineStr">
         <is>
-          <t>value_text</t>
+          <t>value_num</t>
         </is>
       </c>
       <c r="D53" s="21" t="inlineStr">
         <is>
-          <t>결과 판정</t>
+          <t>결과 수치</t>
         </is>
       </c>
       <c r="E53" s="21" t="inlineStr">
         <is>
-          <t>varchar(200)</t>
+          <t>decimal(12,3)</t>
         </is>
       </c>
       <c r="F53" s="22" t="n"/>
@@ -11201,8 +11281,60 @@
       </c>
       <c r="N53" s="21" t="n"/>
     </row>
+    <row r="54">
+      <c r="A54" s="20" t="inlineStr">
+        <is>
+          <t>checkup_results</t>
+        </is>
+      </c>
+      <c r="B54" s="21" t="inlineStr">
+        <is>
+          <t>건강검진 결과 (보류)</t>
+        </is>
+      </c>
+      <c r="C54" s="21" t="inlineStr">
+        <is>
+          <t>value_text</t>
+        </is>
+      </c>
+      <c r="D54" s="21" t="inlineStr">
+        <is>
+          <t>결과 판정</t>
+        </is>
+      </c>
+      <c r="E54" s="21" t="inlineStr">
+        <is>
+          <t>varchar(200)</t>
+        </is>
+      </c>
+      <c r="F54" s="22" t="n"/>
+      <c r="G54" s="21" t="n"/>
+      <c r="H54" s="22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I54" s="21" t="n"/>
+      <c r="J54" s="21" t="n"/>
+      <c r="K54" s="21" t="inlineStr">
+        <is>
+          <t>REQ-015</t>
+        </is>
+      </c>
+      <c r="L54" s="22" t="inlineStr">
+        <is>
+          <t>수정</t>
+        </is>
+      </c>
+      <c r="M54" s="22" t="inlineStr">
+        <is>
+          <t>v1.0</t>
+        </is>
+      </c>
+      <c r="N54" s="21" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:N51"/>
+  <autoFilter ref="A4:N52"/>
   <dataValidations count="3">
     <dataValidation sqref="H5:H300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>

</xml_diff>